<commit_message>
Respaldo automático: cotización COT-2026-001
</commit_message>
<xml_diff>
--- a/Sistema_Inventario_NEMET_Final.xlsx
+++ b/Sistema_Inventario_NEMET_Final.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Cotizador_Rendimientos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Cat_Productos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Clientes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Historial_Cotizaciones" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6243,8 +6244,72 @@
           <t>luismerelles@gmail.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Detalle_Productos</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>COT-2026-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-28 12:49:26</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cliente General</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>13x EPO-DEEP TRANSPARENTE (1.420 kg) [16.00 m² x 1 mm]</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>10010</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Respaldo automático: cotización COT-2026-002
</commit_message>
<xml_diff>
--- a/Sistema_Inventario_NEMET_Final.xlsx
+++ b/Sistema_Inventario_NEMET_Final.xlsx
@@ -6256,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6311,6 +6311,31 @@
         <v>10010</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>COT-2026-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-28 13:58:48</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Luis Manuel Merelles Lourido</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2x EPO-DEEP TRANSPARENTE (7.100 kg) [12.00 m² x 1 mm]</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>7110</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
inventario: asigna SKUs únicos a Epoxy-Mica y Epo-Paint
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Sistema_Inventario_NEMET_Final.xlsx
+++ b/Sistema_Inventario_NEMET_Final.xlsx
@@ -3539,7 +3539,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>EM 01</t>
+          <t>EMI 01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3594,7 +3594,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>EM 02</t>
+          <t>EMI 02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3759,7 +3759,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>EP 01</t>
+          <t>EPA 01</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">

</xml_diff>

<commit_message>
Actualizar precios con lista nueva del proveedor
- Precios de venta al publico sugerido (resinas +5.8%, tintas, pastas, hojuelas)
- PrecioCompra capturado en 57 SKUs (costo con IVA del proveedor)
- Lijadora de piso: $3,999 (antes $0, pendiente)
- 12 SKUs nuevos: Cascara de Naranja, Estuco Veneciano, Grano Wall, Epoxy Cuarzo, Spikes Premium
- Hojuelas re-estructuradas a 2 escalas (0-59.999 kg / +60 kg)
- Hojas Inventario y Cat_Productos sincronizadas (0 diferencias)
- Reporte comparativo completo en comparativo_precios_proveedor.md

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Sistema_Inventario_NEMET_Final.xlsx
+++ b/Sistema_Inventario_NEMET_Final.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q80"/>
+  <dimension ref="A1:Q90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,22 +548,22 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>655.87</v>
       </c>
       <c r="K3" t="n">
-        <v>663.7931034482759</v>
+        <v>685.344827586207</v>
       </c>
       <c r="L3" t="n">
-        <v>106.2068965517242</v>
+        <v>109.655172413793</v>
       </c>
       <c r="M3" t="n">
-        <v>770.0000000000001</v>
+        <v>795</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>663.7931034482759</v>
+        <v>685.344827586207</v>
       </c>
     </row>
     <row r="4">
@@ -603,22 +603,22 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1967.61</v>
       </c>
       <c r="K4" t="n">
-        <v>1896.551724137931</v>
+        <v>2056.896551724138</v>
       </c>
       <c r="L4" t="n">
-        <v>303.448275862069</v>
+        <v>329.1034482758619</v>
       </c>
       <c r="M4" t="n">
-        <v>2200</v>
+        <v>2386</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>1896.551724137931</v>
+        <v>2056.896551724138</v>
       </c>
     </row>
     <row r="5">
@@ -658,22 +658,22 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>3015.44</v>
       </c>
       <c r="K5" t="n">
-        <v>3064.655172413793</v>
+        <v>3182.758620689655</v>
       </c>
       <c r="L5" t="n">
-        <v>490.3448275862069</v>
+        <v>509.2413793103447</v>
       </c>
       <c r="M5" t="n">
-        <v>3555</v>
+        <v>3692</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>3064.655172413793</v>
+        <v>3182.758620689655</v>
       </c>
     </row>
     <row r="6">
@@ -713,22 +713,22 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>6635.89</v>
       </c>
       <c r="K6" t="n">
-        <v>7107.758620689656</v>
+        <v>7344.827586206897</v>
       </c>
       <c r="L6" t="n">
-        <v>1137.241379310345</v>
+        <v>1175.172413793103</v>
       </c>
       <c r="M6" t="n">
-        <v>8245</v>
+        <v>8520</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>7107.758620689656</v>
+        <v>7344.827586206897</v>
       </c>
     </row>
     <row r="7">
@@ -768,22 +768,22 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>784.48</v>
       </c>
       <c r="K7" t="n">
-        <v>818.9655172413794</v>
+        <v>827.5862068965517</v>
       </c>
       <c r="L7" t="n">
-        <v>131.0344827586207</v>
+        <v>132.4137931034483</v>
       </c>
       <c r="M7" t="n">
-        <v>950.0000000000001</v>
+        <v>960</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>818.9655172413794</v>
+        <v>827.5862068965517</v>
       </c>
     </row>
     <row r="8">
@@ -823,22 +823,22 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>2241.3</v>
       </c>
       <c r="K8" t="n">
-        <v>2331.896551724138</v>
+        <v>2379.310344827587</v>
       </c>
       <c r="L8" t="n">
-        <v>373.1034482758621</v>
+        <v>380.6896551724135</v>
       </c>
       <c r="M8" t="n">
-        <v>2705</v>
+        <v>2760</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>2331.896551724138</v>
+        <v>2379.310344827587</v>
       </c>
     </row>
     <row r="9">
@@ -878,22 +878,22 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>3557.7</v>
       </c>
       <c r="K9" t="n">
-        <v>3693.96551724138</v>
+        <v>3793.103448275862</v>
       </c>
       <c r="L9" t="n">
-        <v>591.0344827586208</v>
+        <v>606.8965517241377</v>
       </c>
       <c r="M9" t="n">
-        <v>4285.000000000001</v>
+        <v>4400</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>3693.96551724138</v>
+        <v>3793.103448275862</v>
       </c>
     </row>
     <row r="10">
@@ -933,22 +933,22 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>6186.02</v>
       </c>
       <c r="K10" t="n">
-        <v>6668.103448275862</v>
+        <v>6879.310344827587</v>
       </c>
       <c r="L10" t="n">
-        <v>1066.896551724138</v>
+        <v>1100.689655172413</v>
       </c>
       <c r="M10" t="n">
-        <v>7735</v>
+        <v>7980</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>6668.103448275862</v>
+        <v>6879.310344827587</v>
       </c>
     </row>
     <row r="11">
@@ -988,22 +988,22 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>542.13</v>
       </c>
       <c r="K11" t="n">
-        <v>599.1379310344828</v>
+        <v>620.6896551724138</v>
       </c>
       <c r="L11" t="n">
-        <v>95.86206896551725</v>
+        <v>99.31034482758616</v>
       </c>
       <c r="M11" t="n">
-        <v>695</v>
+        <v>720</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>599.1379310344828</v>
+        <v>620.6896551724138</v>
       </c>
     </row>
     <row r="12">
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1084.26</v>
       </c>
       <c r="K12" t="n">
-        <v>1133.620689655173</v>
+        <v>1241.379310344828</v>
       </c>
       <c r="L12" t="n">
-        <v>181.3793103448277</v>
+        <v>198.6206896551723</v>
       </c>
       <c r="M12" t="n">
-        <v>1315.000000000001</v>
+        <v>1440</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>1133.620689655173</v>
+        <v>1241.379310344828</v>
       </c>
     </row>
     <row r="13">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>2076.12</v>
       </c>
       <c r="K13" t="n">
-        <v>2172.413793103448</v>
+        <v>2379.310344827587</v>
       </c>
       <c r="L13" t="n">
-        <v>347.5862068965517</v>
+        <v>380.6896551724135</v>
       </c>
       <c r="M13" t="n">
-        <v>2520</v>
+        <v>2760</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>2172.413793103448</v>
+        <v>2379.310344827587</v>
       </c>
     </row>
     <row r="14">
@@ -1153,22 +1153,22 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>3329.5</v>
       </c>
       <c r="K14" t="n">
-        <v>3482.758620689655</v>
+        <v>3793.103448275862</v>
       </c>
       <c r="L14" t="n">
-        <v>557.2413793103448</v>
+        <v>606.8965517241377</v>
       </c>
       <c r="M14" t="n">
-        <v>4040</v>
+        <v>4400</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>3482.758620689655</v>
+        <v>3793.103448275862</v>
       </c>
     </row>
     <row r="15">
@@ -1208,22 +1208,22 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>4752</v>
       </c>
       <c r="K15" t="n">
-        <v>5030.172413793104</v>
+        <v>5431.034482758621</v>
       </c>
       <c r="L15" t="n">
-        <v>804.8275862068967</v>
+        <v>868.9655172413786</v>
       </c>
       <c r="M15" t="n">
-        <v>5835.000000000001</v>
+        <v>6300</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>5030.172413793104</v>
+        <v>5431.034482758621</v>
       </c>
     </row>
     <row r="16">
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>6029</v>
       </c>
       <c r="K16" t="n">
-        <v>6456.896551724139</v>
+        <v>6896.551724137931</v>
       </c>
       <c r="L16" t="n">
-        <v>1033.103448275862</v>
+        <v>1103.448275862069</v>
       </c>
       <c r="M16" t="n">
-        <v>7490.000000000001</v>
+        <v>8000</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>6456.896551724139</v>
+        <v>6896.551724137931</v>
       </c>
     </row>
     <row r="17">
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>537.29</v>
       </c>
       <c r="K17" t="n">
         <v>465.5172413793103</v>
@@ -1373,22 +1373,22 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>2927</v>
       </c>
       <c r="K18" t="n">
-        <v>3051.724137931035</v>
+        <v>3275.862068965518</v>
       </c>
       <c r="L18" t="n">
-        <v>488.2758620689656</v>
+        <v>524.1379310344823</v>
       </c>
       <c r="M18" t="n">
-        <v>3540</v>
+        <v>3800</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>3051.724137931035</v>
+        <v>3275.862068965518</v>
       </c>
     </row>
     <row r="19">
@@ -1428,22 +1428,22 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>5533.91</v>
       </c>
       <c r="K19" t="n">
-        <v>5793.103448275862</v>
+        <v>6387.068965517242</v>
       </c>
       <c r="L19" t="n">
-        <v>926.896551724138</v>
+        <v>1021.931034482758</v>
       </c>
       <c r="M19" t="n">
-        <v>6720</v>
+        <v>7409</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>5793.103448275862</v>
+        <v>6387.068965517242</v>
       </c>
     </row>
     <row r="20">
@@ -1483,22 +1483,22 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>522.86</v>
       </c>
       <c r="K20" t="n">
-        <v>530.1724137931035</v>
+        <v>551.7241379310345</v>
       </c>
       <c r="L20" t="n">
-        <v>84.82758620689656</v>
+        <v>88.27586206896547</v>
       </c>
       <c r="M20" t="n">
-        <v>615</v>
+        <v>640</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>530.1724137931035</v>
+        <v>551.7241379310345</v>
       </c>
     </row>
     <row r="21">
@@ -1538,22 +1538,22 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>2608.4</v>
       </c>
       <c r="K21" t="n">
-        <v>2525.862068965517</v>
+        <v>2751.724137931035</v>
       </c>
       <c r="L21" t="n">
-        <v>404.1379310344828</v>
+        <v>440.2758620689651</v>
       </c>
       <c r="M21" t="n">
-        <v>2930</v>
+        <v>3192</v>
       </c>
       <c r="N21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>2525.862068965517</v>
+        <v>2751.724137931035</v>
       </c>
     </row>
     <row r="22">
@@ -1593,22 +1593,22 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>4731.74</v>
       </c>
       <c r="K22" t="n">
-        <v>4814.655172413793</v>
+        <v>5044.827586206897</v>
       </c>
       <c r="L22" t="n">
-        <v>770.3448275862069</v>
+        <v>807.1724137931033</v>
       </c>
       <c r="M22" t="n">
-        <v>5584.999999999999</v>
+        <v>5852</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>4814.655172413793</v>
+        <v>5044.827586206897</v>
       </c>
     </row>
     <row r="23">
@@ -1648,22 +1648,22 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>7813.92</v>
       </c>
       <c r="K23" t="n">
-        <v>8275.862068965518</v>
+        <v>8689.655172413793</v>
       </c>
       <c r="L23" t="n">
-        <v>1324.137931034483</v>
+        <v>1390.344827586207</v>
       </c>
       <c r="M23" t="n">
-        <v>9600.000000000002</v>
+        <v>10080</v>
       </c>
       <c r="N23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>8275.862068965518</v>
+        <v>8689.655172413793</v>
       </c>
     </row>
     <row r="24">
@@ -1929,10 +1929,10 @@
         <v>64.65517241379311</v>
       </c>
       <c r="L28" t="n">
-        <v>10.3448275862069</v>
+        <v>10.34482758620689</v>
       </c>
       <c r="M28" t="n">
-        <v>75.00000000000001</v>
+        <v>75</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
@@ -1981,19 +1981,19 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>99.13793103448276</v>
+        <v>96.55172413793105</v>
       </c>
       <c r="L29" t="n">
-        <v>15.86206896551724</v>
+        <v>15.44827586206895</v>
       </c>
       <c r="M29" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>99.13793103448276</v>
+        <v>96.55172413793105</v>
       </c>
     </row>
     <row r="30">
@@ -2036,19 +2036,19 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>237.0689655172414</v>
+        <v>232.7586206896552</v>
       </c>
       <c r="L30" t="n">
-        <v>37.93103448275863</v>
+        <v>37.24137931034483</v>
       </c>
       <c r="M30" t="n">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>237.0689655172414</v>
+        <v>232.7586206896552</v>
       </c>
     </row>
     <row r="31">
@@ -2091,19 +2091,19 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>456.896551724138</v>
+        <v>448.2758620689655</v>
       </c>
       <c r="L31" t="n">
-        <v>73.10344827586208</v>
+        <v>71.72413793103448</v>
       </c>
       <c r="M31" t="n">
-        <v>530.0000000000001</v>
+        <v>520</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>456.896551724138</v>
+        <v>448.2758620689655</v>
       </c>
     </row>
     <row r="32">
@@ -2146,19 +2146,19 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>732.7586206896552</v>
+        <v>724.1379310344828</v>
       </c>
       <c r="L32" t="n">
-        <v>117.2413793103448</v>
+        <v>115.8620689655172</v>
       </c>
       <c r="M32" t="n">
-        <v>850.0000000000001</v>
+        <v>840</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>732.7586206896552</v>
+        <v>724.1379310344828</v>
       </c>
     </row>
     <row r="33">
@@ -2198,22 +2198,22 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>19.55</v>
       </c>
       <c r="K33" t="n">
-        <v>17.24137931034483</v>
+        <v>21.55172413793104</v>
       </c>
       <c r="L33" t="n">
-        <v>2.758620689655173</v>
+        <v>3.448275862068964</v>
       </c>
       <c r="M33" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>17.24137931034483</v>
+        <v>21.55172413793104</v>
       </c>
     </row>
     <row r="34">
@@ -2253,22 +2253,22 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>53.77</v>
       </c>
       <c r="K34" t="n">
-        <v>51.72413793103448</v>
+        <v>56.03448275862069</v>
       </c>
       <c r="L34" t="n">
-        <v>8.275862068965516</v>
+        <v>8.96551724137931</v>
       </c>
       <c r="M34" t="n">
-        <v>59.99999999999999</v>
+        <v>65</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>51.72413793103448</v>
+        <v>56.03448275862069</v>
       </c>
     </row>
     <row r="35">
@@ -2308,22 +2308,22 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>91.91</v>
       </c>
       <c r="K35" t="n">
-        <v>86.20689655172414</v>
+        <v>94.82758620689656</v>
       </c>
       <c r="L35" t="n">
-        <v>13.79310344827586</v>
+        <v>15.17241379310344</v>
       </c>
       <c r="M35" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>86.20689655172414</v>
+        <v>94.82758620689656</v>
       </c>
     </row>
     <row r="36">
@@ -2363,22 +2363,22 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>161.33</v>
       </c>
       <c r="K36" t="n">
-        <v>155.1724137931035</v>
+        <v>163.7931034482759</v>
       </c>
       <c r="L36" t="n">
-        <v>24.82758620689656</v>
+        <v>26.20689655172413</v>
       </c>
       <c r="M36" t="n">
-        <v>180.0000000000001</v>
+        <v>190</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>155.1724137931035</v>
+        <v>163.7931034482759</v>
       </c>
     </row>
     <row r="37">
@@ -2418,22 +2418,22 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>248.12</v>
       </c>
       <c r="K37" t="n">
-        <v>271.551724137931</v>
+        <v>275.8620689655173</v>
       </c>
       <c r="L37" t="n">
-        <v>43.44827586206896</v>
+        <v>44.13793103448273</v>
       </c>
       <c r="M37" t="n">
-        <v>314.9999999999999</v>
+        <v>320</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>271.551724137931</v>
+        <v>275.8620689655173</v>
       </c>
     </row>
     <row r="38">
@@ -2473,13 +2473,13 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>427.79</v>
       </c>
       <c r="K38" t="n">
         <v>474.1379310344828</v>
       </c>
       <c r="L38" t="n">
-        <v>75.86206896551725</v>
+        <v>75.86206896551721</v>
       </c>
       <c r="M38" t="n">
         <v>550</v>
@@ -2968,13 +2968,13 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>421.06</v>
       </c>
       <c r="K47" t="n">
         <v>431.0344827586207</v>
       </c>
       <c r="L47" t="n">
-        <v>68.96551724137932</v>
+        <v>68.9655172413793</v>
       </c>
       <c r="M47" t="n">
         <v>500</v>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>&lt; 10 kg</t>
+          <t>0 a 59.999 kg</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -3023,22 +3023,22 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>182.7</v>
       </c>
       <c r="K48" t="n">
-        <v>172.4137931034483</v>
+        <v>176.7241379310345</v>
       </c>
       <c r="L48" t="n">
-        <v>27.58620689655173</v>
+        <v>28.27586206896549</v>
       </c>
       <c r="M48" t="n">
-        <v>200.0000000000001</v>
+        <v>205</v>
       </c>
       <c r="N48" t="n">
         <v>0</v>
       </c>
       <c r="Q48" t="n">
-        <v>172.4137931034483</v>
+        <v>176.7241379310345</v>
       </c>
     </row>
     <row r="49">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10 a 20 kg</t>
+          <t>+ 60 kg</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -3078,38 +3078,38 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>182.7</v>
       </c>
       <c r="K49" t="n">
-        <v>168.1034482758621</v>
+        <v>172.4137931034483</v>
       </c>
       <c r="L49" t="n">
-        <v>26.89655172413794</v>
+        <v>27.58620689655172</v>
       </c>
       <c r="M49" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>168.1034482758621</v>
+        <v>172.4137931034483</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>EH 03</t>
+          <t>EHC 01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EPOXY-HOJUELA (1 color)</t>
+          <t xml:space="preserve">EPOXY-HOJUELA (combinación) </t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>25 a 175 kg</t>
+          <t>0 a 59.999 kg</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3133,28 +3133,28 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>214.5</v>
       </c>
       <c r="K50" t="n">
-        <v>159.4827586206897</v>
+        <v>202.5862068965517</v>
       </c>
       <c r="L50" t="n">
-        <v>25.51724137931035</v>
+        <v>32.41379310344826</v>
       </c>
       <c r="M50" t="n">
-        <v>185.0000000000001</v>
+        <v>235</v>
       </c>
       <c r="N50" t="n">
         <v>0</v>
       </c>
       <c r="Q50" t="n">
-        <v>159.4827586206897</v>
+        <v>202.5862068965517</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>EHC 01</t>
+          <t>EHC 02</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>&lt; 10 kg</t>
+          <t>+ 60 kg</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3188,38 +3188,38 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>214.5</v>
       </c>
       <c r="K51" t="n">
-        <v>181.0344827586207</v>
+        <v>198.2758620689655</v>
       </c>
       <c r="L51" t="n">
-        <v>28.96551724137931</v>
+        <v>31.72413793103448</v>
       </c>
       <c r="M51" t="n">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
       </c>
       <c r="Q51" t="n">
-        <v>181.0344827586207</v>
+        <v>198.2758620689655</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>EHC 02</t>
+          <t>EG 01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">EPOXY-HOJUELA (combinación) </t>
+          <t>EPOXY-GRANO</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10 a 20 kg</t>
+          <t>1 a 20 kg</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3246,35 +3246,35 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>176.7241379310345</v>
+        <v>56.03448275862069</v>
       </c>
       <c r="L52" t="n">
-        <v>28.27586206896552</v>
+        <v>8.965517241379311</v>
       </c>
       <c r="M52" t="n">
-        <v>205</v>
+        <v>65</v>
       </c>
       <c r="N52" t="n">
         <v>0</v>
       </c>
       <c r="Q52" t="n">
-        <v>176.7241379310345</v>
+        <v>56.03448275862069</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>EHC 03</t>
+          <t>EG 02</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">EPOXY-HOJUELA (combinación) </t>
+          <t>EPOXY-GRANO</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>25 a 175 kg</t>
+          <t>22.7 a 24.3 kg</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3301,30 +3301,30 @@
         <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>172.4137931034483</v>
+        <v>47.41379310344828</v>
       </c>
       <c r="L53" t="n">
-        <v>27.58620689655173</v>
+        <v>7.586206896551724</v>
       </c>
       <c r="M53" t="n">
-        <v>200.0000000000001</v>
+        <v>55</v>
       </c>
       <c r="N53" t="n">
         <v>0</v>
       </c>
       <c r="Q53" t="n">
-        <v>172.4137931034483</v>
+        <v>47.41379310344828</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>EG 01</t>
+          <t>EGC 01</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EPOXY-GRANO</t>
+          <t>EPOXY-GRANO (combinación)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3356,30 +3356,30 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>56.03448275862069</v>
+        <v>77.58620689655173</v>
       </c>
       <c r="L54" t="n">
-        <v>8.965517241379311</v>
+        <v>12.41379310344828</v>
       </c>
       <c r="M54" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="N54" t="n">
         <v>0</v>
       </c>
       <c r="Q54" t="n">
-        <v>56.03448275862069</v>
+        <v>77.58620689655173</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>EG 02</t>
+          <t>EGC 02</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EPOXY-GRANO</t>
+          <t>EPOXY-GRANO (combinación)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3411,35 +3411,35 @@
         <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>47.41379310344828</v>
+        <v>60.3448275862069</v>
       </c>
       <c r="L55" t="n">
-        <v>7.586206896551724</v>
+        <v>9.655172413793103</v>
       </c>
       <c r="M55" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="N55" t="n">
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>47.41379310344828</v>
+        <v>60.3448275862069</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>EGC 01</t>
+          <t>EMI 01</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EPOXY-GRANO (combinación)</t>
+          <t>EPOXY-MICA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1 a 20 kg</t>
+          <t>1 kg</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3466,35 +3466,35 @@
         <v>0</v>
       </c>
       <c r="K56" t="n">
-        <v>77.58620689655173</v>
+        <v>405.1724137931035</v>
       </c>
       <c r="L56" t="n">
-        <v>12.41379310344828</v>
+        <v>64.82758620689656</v>
       </c>
       <c r="M56" t="n">
-        <v>90</v>
+        <v>470.0000000000001</v>
       </c>
       <c r="N56" t="n">
         <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>77.58620689655173</v>
+        <v>405.1724137931035</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>EGC 02</t>
+          <t>EMI 02</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EPOXY-GRANO (combinación)</t>
+          <t>EPOXY-MICA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>22.7 a 24.3 kg</t>
+          <t>1/2 kg</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3521,30 +3521,30 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>60.3448275862069</v>
+        <v>715.5172413793103</v>
       </c>
       <c r="L57" t="n">
-        <v>9.655172413793103</v>
+        <v>114.4827586206897</v>
       </c>
       <c r="M57" t="n">
-        <v>70</v>
+        <v>830</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
       </c>
       <c r="Q57" t="n">
-        <v>60.3448275862069</v>
+        <v>715.5172413793103</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>EMI 01</t>
+          <t>EMC 01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EPOXY-MICA</t>
+          <t>EPOXY-MICA (combinado)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3576,30 +3576,30 @@
         <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>405.1724137931035</v>
+        <v>426.7241379310345</v>
       </c>
       <c r="L58" t="n">
-        <v>64.82758620689656</v>
+        <v>68.27586206896552</v>
       </c>
       <c r="M58" t="n">
-        <v>470.0000000000001</v>
+        <v>495</v>
       </c>
       <c r="N58" t="n">
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>405.1724137931035</v>
+        <v>426.7241379310345</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>EMI 02</t>
+          <t>EMC 02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EPOXY-MICA</t>
+          <t>EPOXY-MICA (combinado)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3631,36 +3631,34 @@
         <v>0</v>
       </c>
       <c r="K59" t="n">
-        <v>715.5172413793103</v>
+        <v>737.0689655172414</v>
       </c>
       <c r="L59" t="n">
-        <v>114.4827586206897</v>
+        <v>117.9310344827586</v>
       </c>
       <c r="M59" t="n">
-        <v>830</v>
+        <v>855</v>
       </c>
       <c r="N59" t="n">
         <v>0</v>
       </c>
       <c r="Q59" t="n">
-        <v>715.5172413793103</v>
+        <v>737.0689655172414</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>EMC 01</t>
+          <t>EPA 01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EPOXY-MICA (combinado)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>1 kg</t>
-        </is>
+          <t>EPO-PAINT (A y B)</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
       </c>
       <c r="D60" t="n">
         <v>5</v>
@@ -3686,36 +3684,34 @@
         <v>0</v>
       </c>
       <c r="K60" t="n">
-        <v>426.7241379310345</v>
+        <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>68.27586206896552</v>
+        <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>495</v>
+        <v>0</v>
       </c>
       <c r="N60" t="n">
         <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>426.7241379310345</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>EMC 02</t>
+          <t>AS 01</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EPOXY-MICA (combinado)</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>1/2 kg</t>
-        </is>
+          <t>ARENA SILICA</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
       </c>
       <c r="D61" t="n">
         <v>5</v>
@@ -3741,34 +3737,36 @@
         <v>0</v>
       </c>
       <c r="K61" t="n">
-        <v>737.0689655172414</v>
+        <v>0</v>
       </c>
       <c r="L61" t="n">
-        <v>117.9310344827586</v>
+        <v>0</v>
       </c>
       <c r="M61" t="n">
-        <v>855</v>
+        <v>0</v>
       </c>
       <c r="N61" t="n">
         <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>737.0689655172414</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>EPA 01</t>
+          <t>RP 01</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EPO-PAINT (A y B)</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>0</v>
+          <t>RODILLO DE PICOS EPOXY-PISOS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1 Pz</t>
+        </is>
       </c>
       <c r="D62" t="n">
         <v>5</v>
@@ -3791,37 +3789,39 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>474.06</v>
       </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>426.7241379310345</v>
       </c>
       <c r="L62" t="n">
-        <v>0</v>
+        <v>68.27586206896547</v>
       </c>
       <c r="M62" t="n">
-        <v>0</v>
+        <v>495</v>
       </c>
       <c r="N62" t="n">
         <v>0</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
+        <v>426.7241379310345</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AS 01</t>
+          <t>JEP 01</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ARENA SILICA</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>0</v>
+          <t>JALADOR EPÓXICO PREMIUM</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1 Pz</t>
+        </is>
       </c>
       <c r="D63" t="n">
         <v>5</v>
@@ -3844,33 +3844,33 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>406.09</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>366.3793103448277</v>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
+        <v>58.62068965517238</v>
       </c>
       <c r="M63" t="n">
-        <v>0</v>
+        <v>425.0000000000001</v>
       </c>
       <c r="N63" t="n">
         <v>0</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
+        <v>366.3793103448277</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RP 01</t>
+          <t>JEE 01</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>RODILLO DE PICOS EPOXY-PISOS</t>
+          <t>JALADOR PARA EPÓXICOS ECO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3899,33 +3899,33 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="K64" t="n">
-        <v>426.7241379310345</v>
+        <v>64.65517241379312</v>
       </c>
       <c r="L64" t="n">
-        <v>68.27586206896552</v>
+        <v>10.34482758620689</v>
       </c>
       <c r="M64" t="n">
-        <v>495</v>
+        <v>75.00000000000001</v>
       </c>
       <c r="N64" t="n">
         <v>0</v>
       </c>
       <c r="Q64" t="n">
-        <v>426.7241379310345</v>
+        <v>64.65517241379312</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>JEP 01</t>
+          <t>JNE 01</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>JALADOR EPÓXICO PREMIUM</t>
+          <t>JALADOR NIVELADOR EPÓXICO</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3957,30 +3957,30 @@
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>366.3793103448276</v>
+        <v>1370.689655172414</v>
       </c>
       <c r="L65" t="n">
-        <v>58.62068965517242</v>
+        <v>219.3103448275862</v>
       </c>
       <c r="M65" t="n">
-        <v>425.0000000000001</v>
+        <v>1590</v>
       </c>
       <c r="N65" t="n">
         <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>366.3793103448276</v>
+        <v>1370.689655172414</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>JEE 01</t>
+          <t>JD 01</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>JALADOR PARA EPÓXICOS ECO</t>
+          <t>JALADOR DENTADO</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4009,33 +4009,33 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>370.51</v>
       </c>
       <c r="K66" t="n">
-        <v>64.65517241379311</v>
+        <v>336.2068965517242</v>
       </c>
       <c r="L66" t="n">
-        <v>10.3448275862069</v>
+        <v>53.79310344827587</v>
       </c>
       <c r="M66" t="n">
-        <v>75.00000000000001</v>
+        <v>390.0000000000001</v>
       </c>
       <c r="N66" t="n">
         <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>64.65517241379311</v>
+        <v>336.2068965517242</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>JNE 01</t>
+          <t>CV 01</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>JALADOR NIVELADOR EPÓXICO</t>
+          <t>CUÑA PARA VINIL</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4064,33 +4064,33 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>62.71</v>
       </c>
       <c r="K67" t="n">
-        <v>1370.689655172414</v>
+        <v>56.03448275862069</v>
       </c>
       <c r="L67" t="n">
-        <v>219.3103448275862</v>
+        <v>8.96551724137931</v>
       </c>
       <c r="M67" t="n">
-        <v>1590</v>
+        <v>65</v>
       </c>
       <c r="N67" t="n">
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>1370.689655172414</v>
+        <v>56.03448275862069</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>JD 01</t>
+          <t>R 01</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>JALADOR DENTADO</t>
+          <t>RODILLO 4"</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4119,33 +4119,33 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>77.92</v>
       </c>
       <c r="K68" t="n">
-        <v>336.2068965517242</v>
+        <v>68.96551724137932</v>
       </c>
       <c r="L68" t="n">
-        <v>53.79310344827587</v>
+        <v>11.03448275862068</v>
       </c>
       <c r="M68" t="n">
-        <v>390.0000000000001</v>
+        <v>80</v>
       </c>
       <c r="N68" t="n">
         <v>0</v>
       </c>
       <c r="Q68" t="n">
-        <v>336.2068965517242</v>
+        <v>68.96551724137932</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CV 01</t>
+          <t>R 02</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CUÑA PARA VINIL</t>
+          <t>RODILLO 9"</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -4174,33 +4174,33 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>193.32</v>
       </c>
       <c r="K69" t="n">
-        <v>56.03448275862069</v>
+        <v>172.4137931034484</v>
       </c>
       <c r="L69" t="n">
-        <v>8.965517241379311</v>
+        <v>27.58620689655172</v>
       </c>
       <c r="M69" t="n">
-        <v>65</v>
+        <v>200.0000000000001</v>
       </c>
       <c r="N69" t="n">
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>56.03448275862069</v>
+        <v>172.4137931034484</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>R 01</t>
+          <t>F 01</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>RODILLO 4"</t>
+          <t>FELPA 4"</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4229,33 +4229,33 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>38.01</v>
       </c>
       <c r="K70" t="n">
-        <v>68.96551724137932</v>
+        <v>34.48275862068966</v>
       </c>
       <c r="L70" t="n">
-        <v>11.03448275862069</v>
+        <v>5.517241379310342</v>
       </c>
       <c r="M70" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="N70" t="n">
         <v>0</v>
       </c>
       <c r="Q70" t="n">
-        <v>68.96551724137932</v>
+        <v>34.48275862068966</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>R 02</t>
+          <t>F 02</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>RODILLO 9"</t>
+          <t>FELPA 9"</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4284,33 +4284,33 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>133.02</v>
       </c>
       <c r="K71" t="n">
-        <v>172.4137931034483</v>
+        <v>120.6896551724138</v>
       </c>
       <c r="L71" t="n">
-        <v>27.58620689655173</v>
+        <v>19.31034482758619</v>
       </c>
       <c r="M71" t="n">
-        <v>200.0000000000001</v>
+        <v>140</v>
       </c>
       <c r="N71" t="n">
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>172.4137931034483</v>
+        <v>120.6896551724138</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>F 01</t>
+          <t>M 01</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>FELPA 4"</t>
+          <t>MEZCLADOR</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4342,30 +4342,30 @@
         <v>0</v>
       </c>
       <c r="K72" t="n">
-        <v>34.48275862068966</v>
+        <v>163.7931034482759</v>
       </c>
       <c r="L72" t="n">
-        <v>5.517241379310345</v>
+        <v>26.20689655172415</v>
       </c>
       <c r="M72" t="n">
-        <v>40</v>
+        <v>190.0000000000001</v>
       </c>
       <c r="N72" t="n">
         <v>0</v>
       </c>
       <c r="Q72" t="n">
-        <v>34.48275862068966</v>
+        <v>163.7931034482759</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>F 02</t>
+          <t>ES 01</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>FELPA 9"</t>
+          <t>EPOXI SPIKES UNITALLA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4394,33 +4394,33 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>660.26</v>
       </c>
       <c r="K73" t="n">
-        <v>120.6896551724138</v>
+        <v>599.1379310344828</v>
       </c>
       <c r="L73" t="n">
-        <v>19.31034482758621</v>
+        <v>95.86206896551721</v>
       </c>
       <c r="M73" t="n">
-        <v>140</v>
+        <v>695</v>
       </c>
       <c r="N73" t="n">
         <v>0</v>
       </c>
       <c r="Q73" t="n">
-        <v>120.6896551724138</v>
+        <v>599.1379310344828</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>M 01</t>
+          <t>KB 01</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MEZCLADOR</t>
+          <t>KIT DE BORLAS PARA PULIMENTO</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -4449,33 +4449,33 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>418</v>
       </c>
       <c r="K74" t="n">
-        <v>163.7931034482759</v>
+        <v>379.3103448275862</v>
       </c>
       <c r="L74" t="n">
-        <v>26.20689655172415</v>
+        <v>60.68965517241378</v>
       </c>
       <c r="M74" t="n">
-        <v>190.0000000000001</v>
+        <v>440</v>
       </c>
       <c r="N74" t="n">
         <v>0</v>
       </c>
       <c r="Q74" t="n">
-        <v>163.7931034482759</v>
+        <v>379.3103448275862</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ES 01</t>
+          <t>CD 01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EPOXI SPIKES UNITALLA</t>
+          <t>COPA DIAMANTE PARA DESBASTE 7"</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4507,30 +4507,30 @@
         <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>599.1379310344828</v>
+        <v>1650.862068965517</v>
       </c>
       <c r="L75" t="n">
-        <v>95.86206896551725</v>
+        <v>264.1379310344827</v>
       </c>
       <c r="M75" t="n">
-        <v>695</v>
+        <v>1915</v>
       </c>
       <c r="N75" t="n">
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>599.1379310344828</v>
+        <v>1650.862068965517</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>KB 01</t>
+          <t>EB 01</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>KIT DE BORLAS PARA PULIMENTO</t>
+          <t>EPOXI BUBLES</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4559,33 +4559,33 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>0</v>
+        <v>74.81</v>
       </c>
       <c r="K76" t="n">
-        <v>379.3103448275862</v>
+        <v>77.58620689655173</v>
       </c>
       <c r="L76" t="n">
-        <v>60.68965517241379</v>
+        <v>12.41379310344827</v>
       </c>
       <c r="M76" t="n">
-        <v>440</v>
+        <v>90</v>
       </c>
       <c r="N76" t="n">
         <v>0</v>
       </c>
       <c r="Q76" t="n">
-        <v>379.3103448275862</v>
+        <v>77.58620689655173</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CD 01</t>
+          <t>BD 01</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>COPA DIAMANTE PARA DESBASTE 7"</t>
+          <t>BÁSCULA DIGITAL CAPACIDAD 5kg</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4617,30 +4617,30 @@
         <v>0</v>
       </c>
       <c r="K77" t="n">
-        <v>1650.862068965517</v>
+        <v>215.5172413793103</v>
       </c>
       <c r="L77" t="n">
-        <v>264.1379310344827</v>
+        <v>34.48275862068964</v>
       </c>
       <c r="M77" t="n">
-        <v>1915</v>
+        <v>249.9999999999999</v>
       </c>
       <c r="N77" t="n">
         <v>0</v>
       </c>
       <c r="Q77" t="n">
-        <v>1650.862068965517</v>
+        <v>215.5172413793103</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>EB 01</t>
+          <t>LPE 01</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EPOXI BUBLES</t>
+          <t>LIJADORA DE PISO ELÉCTRICA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4669,38 +4669,38 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>0</v>
+        <v>3452.64</v>
       </c>
       <c r="K78" t="n">
-        <v>77.58620689655173</v>
+        <v>3447.413793103448</v>
       </c>
       <c r="L78" t="n">
-        <v>12.41379310344828</v>
+        <v>551.5862068965516</v>
       </c>
       <c r="M78" t="n">
-        <v>90</v>
+        <v>3999</v>
       </c>
       <c r="N78" t="n">
         <v>0</v>
       </c>
       <c r="Q78" t="n">
-        <v>77.58620689655173</v>
+        <v>3447.413793103448</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BD 01</t>
+          <t>CN 01</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BÁSCULA DIGITAL CAPACIDAD 5kg</t>
+          <t>CÁSCARA DE NARANJA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1 Pz</t>
+          <t>0 a 3.999 kg</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4724,77 +4724,627 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>0</v>
+        <v>444.45</v>
       </c>
       <c r="K79" t="n">
-        <v>215.5172413793103</v>
+        <v>500.0000000000001</v>
       </c>
       <c r="L79" t="n">
-        <v>34.48275862068964</v>
+        <v>79.99999999999994</v>
       </c>
       <c r="M79" t="n">
-        <v>249.9999999999999</v>
+        <v>580</v>
       </c>
       <c r="N79" t="n">
         <v>0</v>
       </c>
       <c r="Q79" t="n">
-        <v>215.5172413793103</v>
+        <v>500.0000000000001</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>LPE 01</t>
+          <t>CN 02</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>LIJADORA DE PISO ELÉCTRICA</t>
+          <t>CÁSCARA DE NARANJA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
+          <t>4 a 7.999 kg</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>433.74</v>
+      </c>
+      <c r="K80" t="n">
+        <v>482.7586206896552</v>
+      </c>
+      <c r="L80" t="n">
+        <v>77.24137931034477</v>
+      </c>
+      <c r="M80" t="n">
+        <v>560</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>482.7586206896552</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>CN 03</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>CÁSCARA DE NARANJA</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>8 a 19.999 kg</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>423.54</v>
+      </c>
+      <c r="K81" t="n">
+        <v>465.5172413793103</v>
+      </c>
+      <c r="L81" t="n">
+        <v>74.48275862068965</v>
+      </c>
+      <c r="M81" t="n">
+        <v>540</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>465.5172413793103</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>CN 04</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>CÁSCARA DE NARANJA</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>+ 20 kg</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>5</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>413.8</v>
+      </c>
+      <c r="K82" t="n">
+        <v>448.2758620689655</v>
+      </c>
+      <c r="L82" t="n">
+        <v>71.72413793103448</v>
+      </c>
+      <c r="M82" t="n">
+        <v>520</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>448.2758620689655</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ESV 01</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ESTUCO VENECIANO</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>1 L</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>5</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>400</v>
+      </c>
+      <c r="K83" t="n">
+        <v>413.7931034482759</v>
+      </c>
+      <c r="L83" t="n">
+        <v>66.20689655172413</v>
+      </c>
+      <c r="M83" t="n">
+        <v>480</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>413.7931034482759</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ESV 02</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ESTUCO VENECIANO</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>4 L</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>5</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>380</v>
+      </c>
+      <c r="K84" t="n">
+        <v>396.551724137931</v>
+      </c>
+      <c r="L84" t="n">
+        <v>63.44827586206895</v>
+      </c>
+      <c r="M84" t="n">
+        <v>460</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>396.551724137931</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ESV 03</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ESTUCO VENECIANO</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>19 L</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>5</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>361</v>
+      </c>
+      <c r="K85" t="n">
+        <v>379.3103448275862</v>
+      </c>
+      <c r="L85" t="n">
+        <v>60.68965517241378</v>
+      </c>
+      <c r="M85" t="n">
+        <v>440</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>379.3103448275862</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>GW 01</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>GRANO WALL</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>4 L</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>5</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>231.58</v>
+      </c>
+      <c r="K86" t="n">
+        <v>237.0689655172414</v>
+      </c>
+      <c r="L86" t="n">
+        <v>37.93103448275861</v>
+      </c>
+      <c r="M86" t="n">
+        <v>275</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>237.0689655172414</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>GW 02</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>GRANO WALL</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>19 L</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>5</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>182.83</v>
+      </c>
+      <c r="K87" t="n">
+        <v>193.9655172413793</v>
+      </c>
+      <c r="L87" t="n">
+        <v>31.03448275862067</v>
+      </c>
+      <c r="M87" t="n">
+        <v>225</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>193.9655172413793</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>EC 01</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>EPOXY CUARZO</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>0 a 59.999 kg</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>5</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>29.34</v>
+      </c>
+      <c r="K88" t="n">
+        <v>30.17241379310345</v>
+      </c>
+      <c r="L88" t="n">
+        <v>4.827586206896548</v>
+      </c>
+      <c r="M88" t="n">
+        <v>35</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>30.17241379310345</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>EC 02</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>EPOXY CUARZO</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>+ 60 kg</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>5</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>29.34</v>
+      </c>
+      <c r="K89" t="n">
+        <v>25.86206896551724</v>
+      </c>
+      <c r="L89" t="n">
+        <v>4.137931034482758</v>
+      </c>
+      <c r="M89" t="n">
+        <v>30</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>25.86206896551724</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ESP 01</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>EPOXY SPIKES PREMIUM</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
           <t>1 Pz</t>
         </is>
       </c>
-      <c r="D80" t="n">
-        <v>5</v>
-      </c>
-      <c r="E80" t="n">
-        <v>0</v>
-      </c>
-      <c r="F80" t="n">
-        <v>0</v>
-      </c>
-      <c r="G80" t="n">
-        <v>0</v>
-      </c>
-      <c r="H80" t="n">
-        <v>0</v>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>⚠️ REABASTECER</t>
-        </is>
-      </c>
-      <c r="J80" t="n">
-        <v>0</v>
-      </c>
-      <c r="K80" t="n">
-        <v>0</v>
-      </c>
-      <c r="L80" t="n">
-        <v>0</v>
-      </c>
-      <c r="M80" t="n">
-        <v>0</v>
-      </c>
-      <c r="N80" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q80" t="n">
-        <v>0</v>
+      <c r="D90" t="n">
+        <v>5</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>⚠️ REABASTECER</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>2373.11</v>
+      </c>
+      <c r="K90" t="n">
+        <v>2153.448275862069</v>
+      </c>
+      <c r="L90" t="n">
+        <v>344.5517241379307</v>
+      </c>
+      <c r="M90" t="n">
+        <v>2498</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>2153.448275862069</v>
       </c>
     </row>
   </sheetData>
@@ -5229,7 +5779,7 @@
         <v>1.5</v>
       </c>
       <c r="D2" t="n">
-        <v>695</v>
+        <v>720</v>
       </c>
       <c r="E2" t="n">
         <v>1.2</v>
@@ -5251,7 +5801,7 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>1315</v>
+        <v>1440</v>
       </c>
       <c r="E3" t="n">
         <v>1.2</v>
@@ -5273,7 +5823,7 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>2520</v>
+        <v>2760</v>
       </c>
       <c r="E4" t="n">
         <v>1.2</v>
@@ -5295,7 +5845,7 @@
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>4040</v>
+        <v>4400</v>
       </c>
       <c r="E5" t="n">
         <v>1.2</v>
@@ -5317,7 +5867,7 @@
         <v>15</v>
       </c>
       <c r="D6" t="n">
-        <v>5835</v>
+        <v>6300</v>
       </c>
       <c r="E6" t="n">
         <v>1.2</v>
@@ -5339,7 +5889,7 @@
         <v>20</v>
       </c>
       <c r="D7" t="n">
-        <v>7490</v>
+        <v>8000</v>
       </c>
       <c r="E7" t="n">
         <v>1.2</v>
@@ -5361,7 +5911,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>950</v>
+        <v>960</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
@@ -5383,7 +5933,7 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>2705</v>
+        <v>2760</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -5405,7 +5955,7 @@
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>4285</v>
+        <v>4400</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -5427,7 +5977,7 @@
         <v>19</v>
       </c>
       <c r="D11" t="n">
-        <v>7735</v>
+        <v>7980</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -5449,7 +5999,7 @@
         <v>1.42</v>
       </c>
       <c r="D12" t="n">
-        <v>770</v>
+        <v>795</v>
       </c>
       <c r="E12" t="n">
         <v>1.07</v>
@@ -5471,7 +6021,7 @@
         <v>4.26</v>
       </c>
       <c r="D13" t="n">
-        <v>2200</v>
+        <v>2386</v>
       </c>
       <c r="E13" t="n">
         <v>1.07</v>
@@ -5493,7 +6043,7 @@
         <v>7.1</v>
       </c>
       <c r="D14" t="n">
-        <v>3555</v>
+        <v>3692</v>
       </c>
       <c r="E14" t="n">
         <v>1.07</v>
@@ -5515,7 +6065,7 @@
         <v>17.04</v>
       </c>
       <c r="D15" t="n">
-        <v>8245</v>
+        <v>8520</v>
       </c>
       <c r="E15" t="n">
         <v>1.07</v>
@@ -5559,7 +6109,7 @@
         <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>3540</v>
+        <v>3800</v>
       </c>
       <c r="E17" t="n">
         <v>0.3333</v>
@@ -5581,7 +6131,7 @@
         <v>20.025</v>
       </c>
       <c r="D18" t="n">
-        <v>6720</v>
+        <v>7409</v>
       </c>
       <c r="E18" t="n">
         <v>0.3333</v>
@@ -5603,7 +6153,7 @@
         <v>1.333</v>
       </c>
       <c r="D19" t="n">
-        <v>615</v>
+        <v>640</v>
       </c>
       <c r="E19" t="n">
         <v>1.07</v>
@@ -5625,7 +6175,7 @@
         <v>6.65</v>
       </c>
       <c r="D20" t="n">
-        <v>2930</v>
+        <v>3192</v>
       </c>
       <c r="E20" t="n">
         <v>1.07</v>
@@ -5647,7 +6197,7 @@
         <v>13.3</v>
       </c>
       <c r="D21" t="n">
-        <v>5585</v>
+        <v>5852</v>
       </c>
       <c r="E21" t="n">
         <v>1.07</v>
@@ -5669,7 +6219,7 @@
         <v>24</v>
       </c>
       <c r="D22" t="n">
-        <v>9600</v>
+        <v>10080</v>
       </c>
       <c r="E22" t="n">
         <v>1.07</v>
@@ -5801,7 +6351,7 @@
         <v>100</v>
       </c>
       <c r="D28" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
@@ -5823,7 +6373,7 @@
         <v>250</v>
       </c>
       <c r="D29" t="n">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
@@ -5845,7 +6395,7 @@
         <v>500</v>
       </c>
       <c r="D30" t="n">
-        <v>530</v>
+        <v>520</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
@@ -5867,7 +6417,7 @@
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>850</v>
+        <v>840</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
@@ -5889,7 +6439,7 @@
         <v>20</v>
       </c>
       <c r="D32" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
@@ -5911,7 +6461,7 @@
         <v>60</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E33" t="n">
         <v>1</v>
@@ -5933,7 +6483,7 @@
         <v>100</v>
       </c>
       <c r="D34" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
@@ -5955,7 +6505,7 @@
         <v>250</v>
       </c>
       <c r="D35" t="n">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="E35" t="n">
         <v>1</v>
@@ -5977,7 +6527,7 @@
         <v>500</v>
       </c>
       <c r="D36" t="n">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="E36" t="n">
         <v>1</v>

</xml_diff>